<commit_message>
Lab Assignment 4 and Lab assignment 3 plotted train vs test for k=1:100
</commit_message>
<xml_diff>
--- a/Data/KNN_Confusion_Matrix.xlsx
+++ b/Data/KNN_Confusion_Matrix.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VSCode\Python\ML-Lab-Assignments\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{78F3A47B-5795-4F7C-8773-558BC632A8AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADC01D8D-0F7B-4B05-93E7-4688B63A5673}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="18105" activeTab="1" xr2:uid="{AFA831A1-7E53-4F9B-BB89-9BDE304F9089}"/>
+    <workbookView xWindow="3225" yWindow="4815" windowWidth="21600" windowHeight="13185" xr2:uid="{AFA831A1-7E53-4F9B-BB89-9BDE304F9089}"/>
   </bookViews>
   <sheets>
-    <sheet name="Training Data" sheetId="1" r:id="rId1"/>
-    <sheet name="Test Data" sheetId="2" r:id="rId2"/>
+    <sheet name="Values" sheetId="1" r:id="rId1"/>
+    <sheet name="CM_Train" sheetId="3" r:id="rId2"/>
+    <sheet name="CM_Test" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,12 +38,30 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="8">
   <si>
     <t>Positive</t>
   </si>
   <si>
     <t>Negative</t>
+  </si>
+  <si>
+    <t>TP</t>
+  </si>
+  <si>
+    <t>TN</t>
+  </si>
+  <si>
+    <t>FP</t>
+  </si>
+  <si>
+    <t>FN</t>
+  </si>
+  <si>
+    <t>Test</t>
+  </si>
+  <si>
+    <t>Train</t>
   </si>
 </sst>
 </file>
@@ -414,6 +433,64 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B08D199-B99C-4D83-B198-7DAA26734C45}">
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2">
+        <v>136</v>
+      </c>
+      <c r="C2">
+        <v>46</v>
+      </c>
+      <c r="D2">
+        <v>62</v>
+      </c>
+      <c r="E2">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3">
+        <v>30</v>
+      </c>
+      <c r="C3">
+        <v>47</v>
+      </c>
+      <c r="D3">
+        <v>41</v>
+      </c>
+      <c r="E3">
+        <v>134</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E692D8A-E9A3-4894-8239-A8116F5E4A2D}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -452,8 +529,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7FF1A95-A9D4-4745-8776-00281719C477}">
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76DBB9CC-05A2-4D23-ADDE-9912CCACEB13}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>

</xml_diff>